<commit_message>
feat(schedule): enforce one primary per shift
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -3082,7 +3082,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3105,7 +3105,7 @@
       <c r="B2" s="2" t="str">
         <v>每日工时上限</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="2" t="str">
         <v>12</v>
       </c>
       <c r="D2" s="2" t="str">
@@ -3119,7 +3119,7 @@
       <c r="B3" s="2" t="str">
         <v>历史统计天数</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="2" t="str">
         <v>7</v>
       </c>
       <c r="D3" s="2" t="str">
@@ -3161,7 +3161,7 @@
       <c r="B6" s="2" t="str">
         <v>连续工作惩罚</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="2" t="str">
         <v>5</v>
       </c>
       <c r="D6" s="2" t="str">
@@ -3189,7 +3189,7 @@
       <c r="B8" s="2" t="str">
         <v>高负荷疲劳阈值</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="2" t="str">
         <v>4</v>
       </c>
       <c r="D8" s="2" t="str">
@@ -3203,7 +3203,7 @@
       <c r="B9" s="2" t="str">
         <v>高负荷恢复分钟</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="2" t="str">
         <v>360</v>
       </c>
       <c r="D9" s="2" t="str">
@@ -3231,7 +3231,7 @@
       <c r="B11" s="2" t="str">
         <v>普通岗位最小衔接间隔</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="2" t="str">
         <v>90</v>
       </c>
       <c r="D11" s="2" t="str">
@@ -3259,7 +3259,7 @@
       <c r="B13" s="2" t="str">
         <v>滚动负荷窗口分钟</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="2" t="str">
         <v>360</v>
       </c>
       <c r="D13" s="2" t="str">
@@ -3273,7 +3273,7 @@
       <c r="B14" s="2" t="str">
         <v>滚动负荷疲劳上限</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="2" t="str">
         <v>8</v>
       </c>
       <c r="D14" s="2" t="str">
@@ -3310,203 +3310,217 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
-        <v>tr121H02CooldownWorkdays</v>
+        <v>dailyPrimaryPositionUniqueEnabled</v>
       </c>
       <c r="B17" s="2" t="str">
-        <v>TR121/H02 冷却工作班数</v>
-      </c>
-      <c r="C17" s="2">
-        <v>3</v>
+        <v>同一班表一号岗位单人限一次</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D17" s="2" t="str">
-        <v>承担 TR121/H02 后优先避开的后续已归档工作班数，0 表示关闭</v>
+        <v>同一张生成班表内，每个人最多承担一次非督导首个岗位；无法安排时保留空岗</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>lateShiftRecoveryEnabled</v>
+        <v>tr121H02CooldownWorkdays</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>启用跨工作日恢复</v>
+        <v>TR121/H02 冷却工作班数</v>
       </c>
       <c r="C18" s="2" t="str">
-        <v>是</v>
+        <v>3</v>
       </c>
       <c r="D18" s="2" t="str">
-        <v>是否保护上一班末班重点岗位人员</v>
+        <v>承担 TR121/H02 后优先避开的后续已归档工作班数，0 表示关闭</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>nextWorkdayRecoveryMode</v>
+        <v>lateShiftRecoveryEnabled</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>跨工作日恢复目标强度</v>
+        <v>启用跨工作日恢复</v>
       </c>
       <c r="C19" s="2" t="str">
-        <v>prefer</v>
+        <v>是</v>
       </c>
       <c r="D19" s="2" t="str">
-        <v>优先避开或严格限制次班恢复目标</v>
+        <v>是否保护上一班末班重点岗位人员</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>lateShiftEndTime</v>
+        <v>nextWorkdayRecoveryMode</v>
       </c>
       <c r="B20" s="2" t="str">
-        <v>末班结束界线</v>
+        <v>跨工作日恢复目标强度</v>
       </c>
       <c r="C20" s="2" t="str">
-        <v>23:00</v>
+        <v>prefer</v>
       </c>
       <c r="D20" s="2" t="str">
-        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
+        <v>优先避开或严格限制次班恢复目标</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
-        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
+        <v>lateShiftEndTime</v>
       </c>
       <c r="B21" s="2" t="str">
-        <v>分队长并行督导最大重叠分钟</v>
-      </c>
-      <c r="C21" s="2">
-        <v>30</v>
+        <v>末班结束界线</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v>23:00</v>
       </c>
       <c r="D21" s="2" t="str">
-        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
+        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="str">
-        <v>dutyFatiguePoints</v>
+        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
       </c>
       <c r="B22" s="2" t="str">
-        <v>值班疲劳点数</v>
-      </c>
-      <c r="C22" s="2">
-        <v>12</v>
+        <v>分队长并行督导最大重叠分钟</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>30</v>
       </c>
       <c r="D22" s="2" t="str">
-        <v>值班任务计入的疲劳点</v>
+        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="str">
-        <v>earlyDepartureCutoffTime</v>
+        <v>dutyFatiguePoints</v>
       </c>
       <c r="B23" s="2" t="str">
-        <v>提前下班截载节点</v>
+        <v>值班疲劳点数</v>
       </c>
       <c r="C23" s="2" t="str">
-        <v>12:00</v>
+        <v>12</v>
       </c>
       <c r="D23" s="2" t="str">
-        <v>严格早于该时间计提前下班</v>
+        <v>值班任务计入的疲劳点</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="str">
-        <v>afternoonRestStartTime</v>
+        <v>earlyDepartureCutoffTime</v>
       </c>
       <c r="B24" s="2" t="str">
-        <v>下午无航班开始</v>
+        <v>提前下班截载节点</v>
       </c>
       <c r="C24" s="2" t="str">
         <v>12:00</v>
       </c>
       <c r="D24" s="2" t="str">
-        <v>下午无航班统计起点</v>
+        <v>严格早于该时间计提前下班</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="str">
-        <v>afternoonRestEndTime</v>
+        <v>afternoonRestStartTime</v>
       </c>
       <c r="B25" s="2" t="str">
-        <v>下午无航班结束</v>
+        <v>下午无航班开始</v>
       </c>
       <c r="C25" s="2" t="str">
-        <v>18:00</v>
+        <v>12:00</v>
       </c>
       <c r="D25" s="2" t="str">
-        <v>下午无航班统计终点</v>
+        <v>下午无航班统计起点</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="str">
-        <v>workloadBalanceEnabled</v>
+        <v>afternoonRestEndTime</v>
       </c>
       <c r="B26" s="2" t="str">
-        <v>启用工时疲劳均衡</v>
+        <v>下午无航班结束</v>
       </c>
       <c r="C26" s="2" t="str">
-        <v>是</v>
+        <v>18:00</v>
       </c>
       <c r="D26" s="2" t="str">
-        <v>是否执行人员负荷均衡</v>
+        <v>下午无航班统计终点</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="str">
-        <v>dailyFlightCountBalanceExemptHalfRest</v>
+        <v>workloadBalanceEnabled</v>
       </c>
       <c r="B27" s="2" t="str">
-        <v>半休人员豁免</v>
+        <v>启用工时疲劳均衡</v>
       </c>
       <c r="C27" s="2" t="str">
         <v>是</v>
       </c>
       <c r="D27" s="2" t="str">
-        <v>勾选后半休人员不参与同一工作班航班数比较</v>
+        <v>是否执行人员负荷均衡</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="str">
-        <v>dailyFlightCountBalanceExemptTeamLeaders</v>
+        <v>dailyFlightCountBalanceExemptHalfRest</v>
       </c>
       <c r="B28" s="2" t="str">
-        <v>分队长豁免</v>
+        <v>半休人员豁免</v>
       </c>
       <c r="C28" s="2" t="str">
         <v>是</v>
       </c>
       <c r="D28" s="2" t="str">
-        <v>勾选后分队长不参与同一工作班航班数比较</v>
+        <v>勾选后半休人员不参与同一工作班航班数比较</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="str">
-        <v>maxWorkHoursDifference</v>
+        <v>dailyFlightCountBalanceExemptTeamLeaders</v>
       </c>
       <c r="B29" s="2" t="str">
-        <v>最大工时差</v>
-      </c>
-      <c r="C29" s="2">
-        <v>2</v>
+        <v>分队长豁免</v>
+      </c>
+      <c r="C29" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D29" s="2" t="str">
-        <v>常规人员当日工时差目标</v>
+        <v>勾选后分队长不参与同一工作班航班数比较</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="str">
+        <v>maxWorkHoursDifference</v>
+      </c>
+      <c r="B30" s="2" t="str">
+        <v>最大工时差</v>
+      </c>
+      <c r="C30" s="2" t="str">
+        <v>2</v>
+      </c>
+      <c r="D30" s="2" t="str">
+        <v>常规人员当日工时差目标</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="str">
         <v>maxTodayFatigueDifference</v>
       </c>
-      <c r="B30" s="2" t="str">
+      <c r="B31" s="2" t="str">
         <v>最大当日疲劳差</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C31" s="2" t="str">
         <v>4</v>
       </c>
-      <c r="D30" s="2" t="str">
+      <c r="D31" s="2" t="str">
         <v>常规人员当日疲劳差目标</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>